<commit_message>
Custom user model enhancement
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A2760CB-A687-4D3D-8402-EBA2759068E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6676C34C-0877-4616-AFB4-3F61606B564F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>username</t>
   </si>
@@ -36,9 +36,6 @@
     <t>role</t>
   </si>
   <si>
-    <t>mina</t>
-  </si>
-  <si>
     <t>مخدوم</t>
   </si>
   <si>
@@ -55,6 +52,21 @@
   </si>
   <si>
     <t>Trumpet_1</t>
+  </si>
+  <si>
+    <t>full_name</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>whatsapp</t>
+  </si>
+  <si>
+    <t>فريد فايز</t>
   </si>
 </sst>
 </file>
@@ -104,11 +116,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -399,56 +408,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.88671875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="2" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding users families and satges
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6676C34C-0877-4616-AFB4-3F61606B564F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49676176-89D8-4D31-875A-FC9A0D0473FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="2610" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ورقة1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="81">
   <si>
     <t>username</t>
   </si>
@@ -39,18 +39,6 @@
     <t>مخدوم</t>
   </si>
   <si>
-    <t>john</t>
-  </si>
-  <si>
-    <t>خادم عادي</t>
-  </si>
-  <si>
-    <t>peter</t>
-  </si>
-  <si>
-    <t>امين اسرة</t>
-  </si>
-  <si>
     <t>Trumpet_1</t>
   </si>
   <si>
@@ -63,10 +51,223 @@
     <t>phone</t>
   </si>
   <si>
-    <t>whatsapp</t>
-  </si>
-  <si>
-    <t>فريد فايز</t>
+    <t>D27-0001</t>
+  </si>
+  <si>
+    <t>D27-0002</t>
+  </si>
+  <si>
+    <t>D27-0003</t>
+  </si>
+  <si>
+    <t>D27-0004</t>
+  </si>
+  <si>
+    <t>D27-0005</t>
+  </si>
+  <si>
+    <t>D27-0006</t>
+  </si>
+  <si>
+    <t>D27-0007</t>
+  </si>
+  <si>
+    <t>D27-0008</t>
+  </si>
+  <si>
+    <t>D27-0009</t>
+  </si>
+  <si>
+    <t>D27-0010</t>
+  </si>
+  <si>
+    <t>D27-0011</t>
+  </si>
+  <si>
+    <t>D27-0012</t>
+  </si>
+  <si>
+    <t>D27-0013</t>
+  </si>
+  <si>
+    <t>D27-0014</t>
+  </si>
+  <si>
+    <t>D27-0015</t>
+  </si>
+  <si>
+    <t>D27-0016</t>
+  </si>
+  <si>
+    <t>D27-0017</t>
+  </si>
+  <si>
+    <t>D27-0018</t>
+  </si>
+  <si>
+    <t>D27-0019</t>
+  </si>
+  <si>
+    <t>D27-0020</t>
+  </si>
+  <si>
+    <t>Trumpet_10</t>
+  </si>
+  <si>
+    <t>Trumpet_11</t>
+  </si>
+  <si>
+    <t>Trumpet_12</t>
+  </si>
+  <si>
+    <t>Trumpet_13</t>
+  </si>
+  <si>
+    <t>Trumpet_14</t>
+  </si>
+  <si>
+    <t>Trumpet_15</t>
+  </si>
+  <si>
+    <t>Trumpet_16</t>
+  </si>
+  <si>
+    <t>Trumpet_17</t>
+  </si>
+  <si>
+    <t>Trumpet_18</t>
+  </si>
+  <si>
+    <t>محمد أحمد علي</t>
+  </si>
+  <si>
+    <t>محمود حسن إبراهيم</t>
+  </si>
+  <si>
+    <t>أحمد مصطفى محمود</t>
+  </si>
+  <si>
+    <t>يوسف خالد عبد الله</t>
+  </si>
+  <si>
+    <t>عمر سامي حسين</t>
+  </si>
+  <si>
+    <t>كريم طارق عبد الرحمن</t>
+  </si>
+  <si>
+    <t>عبد الله محمد حسن</t>
+  </si>
+  <si>
+    <t>مينا فؤاد جرجس</t>
+  </si>
+  <si>
+    <t>بيتر مجدي كامل</t>
+  </si>
+  <si>
+    <t>جورج سامح فؤاد</t>
+  </si>
+  <si>
+    <t>شادي نبيل عادل</t>
+  </si>
+  <si>
+    <t>رامي ممدوح صبحي</t>
+  </si>
+  <si>
+    <t>هاني عاطف مراد</t>
+  </si>
+  <si>
+    <t>تامر وجدي أنور</t>
+  </si>
+  <si>
+    <t>إيهاب سمير جلال</t>
+  </si>
+  <si>
+    <t>عماد زكريا شوقي</t>
+  </si>
+  <si>
+    <t>حسام الدين محمد</t>
+  </si>
+  <si>
+    <t>وائل لطفي عبد المسيح</t>
+  </si>
+  <si>
+    <t>سامي نجيب حنا</t>
+  </si>
+  <si>
+    <t>فادي ماهر بشاي</t>
+  </si>
+  <si>
+    <t>12 شارع النيل، المعادي، القاهرة</t>
+  </si>
+  <si>
+    <t>45 شارع الهرم، الجيزة</t>
+  </si>
+  <si>
+    <t>8 شارع التحرير، الدقي، الجيزة</t>
+  </si>
+  <si>
+    <t>23 شارع فيصل، الطالبية، الجيزة</t>
+  </si>
+  <si>
+    <t>67 شارع السودان، المهندسين، الجيزة</t>
+  </si>
+  <si>
+    <t>14 شارع جامعة الدول العربية، المهندسين</t>
+  </si>
+  <si>
+    <t>9 شارع القصر العيني، وسط البلد، القاهرة</t>
+  </si>
+  <si>
+    <t>31 شارع عباس العقاد، مدينة نصر، القاهرة</t>
+  </si>
+  <si>
+    <t>5 شارع مصطفى النحاس، مدينة نصر</t>
+  </si>
+  <si>
+    <t>18 شارع الخليفة المأمون، مصر الجديدة</t>
+  </si>
+  <si>
+    <t>27 شارع جسر السويس، القاهرة</t>
+  </si>
+  <si>
+    <t>6 شارع عين شمس، القاهرة</t>
+  </si>
+  <si>
+    <t>40 شارع شبرا، روض الفرج، القاهرة</t>
+  </si>
+  <si>
+    <t>11 شارع الترعة البولاقية، شبرا</t>
+  </si>
+  <si>
+    <t>29 شارع كورنيش النيل، الزمالك</t>
+  </si>
+  <si>
+    <t>3 شارع أحمد عرابي، المهندسين</t>
+  </si>
+  <si>
+    <t>22 شارع الطيران، مدينة نصر</t>
+  </si>
+  <si>
+    <t>10 شارع النزهة، مصر الجديدة</t>
+  </si>
+  <si>
+    <t>16 شارع الحجاز، مصر الجديدة</t>
+  </si>
+  <si>
+    <t>7 شارع الهرم القديم، الجيزة</t>
+  </si>
+  <si>
+    <t>stage</t>
+  </si>
+  <si>
+    <t>family</t>
+  </si>
+  <si>
+    <t>اسرة القديس اسطفانوس</t>
+  </si>
+  <si>
+    <t>المرحلة الاولي</t>
   </si>
 </sst>
 </file>
@@ -408,19 +609,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.88671875" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -431,49 +633,539 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2">
+        <v>1012345678</v>
+      </c>
+      <c r="G2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="B3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>58</v>
+      </c>
+      <c r="F3">
+        <v>1023456789</v>
+      </c>
+      <c r="G3" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="B4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4">
+        <v>1034567890</v>
+      </c>
+      <c r="G4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5">
+        <v>1112345678</v>
+      </c>
+      <c r="G5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="B6" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6">
+        <v>1123456789</v>
+      </c>
+      <c r="G6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>7</v>
+      <c r="C7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7">
+        <v>1134567890</v>
+      </c>
+      <c r="G7" t="s">
+        <v>79</v>
+      </c>
+      <c r="H7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8">
+        <v>1212345678</v>
+      </c>
+      <c r="G8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" t="s">
+        <v>64</v>
+      </c>
+      <c r="F9">
+        <v>1223456789</v>
+      </c>
+      <c r="G9" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" t="s">
+        <v>45</v>
+      </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10">
+        <v>1234567890</v>
+      </c>
+      <c r="G10" t="s">
+        <v>79</v>
+      </c>
+      <c r="H10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" t="s">
+        <v>66</v>
+      </c>
+      <c r="F11">
+        <v>1512345678</v>
+      </c>
+      <c r="G11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12">
+        <v>1523456789</v>
+      </c>
+      <c r="G12" t="s">
+        <v>79</v>
+      </c>
+      <c r="H12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13">
+        <v>1534567890</v>
+      </c>
+      <c r="G13" t="s">
+        <v>79</v>
+      </c>
+      <c r="H13" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D14" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14">
+        <v>1045678901</v>
+      </c>
+      <c r="G14" t="s">
+        <v>79</v>
+      </c>
+      <c r="H14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E15" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15">
+        <v>1145678901</v>
+      </c>
+      <c r="G15" t="s">
+        <v>79</v>
+      </c>
+      <c r="H15" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E16" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16">
+        <v>1245678901</v>
+      </c>
+      <c r="G16" t="s">
+        <v>79</v>
+      </c>
+      <c r="H16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17">
+        <v>1545678901</v>
+      </c>
+      <c r="G17" t="s">
+        <v>79</v>
+      </c>
+      <c r="H17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D18" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F18">
+        <v>1056789012</v>
+      </c>
+      <c r="G18" t="s">
+        <v>79</v>
+      </c>
+      <c r="H18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19">
+        <v>1156789012</v>
+      </c>
+      <c r="G19" t="s">
+        <v>79</v>
+      </c>
+      <c r="H19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20">
+        <v>1256789012</v>
+      </c>
+      <c r="G20" t="s">
+        <v>79</v>
+      </c>
+      <c r="H20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21">
+        <v>1556789012</v>
+      </c>
+      <c r="G21" t="s">
+        <v>79</v>
+      </c>
+      <c r="H21" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove service account key
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\marmina\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE84492-72BE-49F1-9415-6BB7C2A0119C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{220DB113-A717-4D0F-837B-2838F0DFBF43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="44">
   <si>
     <t>username</t>
   </si>
@@ -148,6 +148,15 @@
   </si>
   <si>
     <t>اسرة البابا اثناسيوس</t>
+  </si>
+  <si>
+    <t>D20-0001</t>
+  </si>
+  <si>
+    <t>مخدوم</t>
+  </si>
+  <si>
+    <t>ديفيد نادر نبيه</t>
   </si>
 </sst>
 </file>
@@ -823,7 +832,24 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B13"/>
+      <c r="A13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B14"/>

</xml_diff>